<commit_message>
organizar mapas y labels de municipios
</commit_message>
<xml_diff>
--- a/03_Outputs/Consolidada_ref_subset/04_Cluster/Summary_Stats.xlsx
+++ b/03_Outputs/Consolidada_ref_subset/04_Cluster/Summary_Stats.xlsx
@@ -406,7 +406,7 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>5.523024430475022E-17</v>
+        <v>5.521545972967087E-17</v>
       </c>
       <c r="E2">
         <v>0.9999999999999999</v>
@@ -433,7 +433,7 @@
         <v>22</v>
       </c>
       <c r="D3">
-        <v>2.459167654864849E-18</v>
+        <v>2.491200900870102E-18</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -460,7 +460,7 @@
         <v>22</v>
       </c>
       <c r="D4">
-        <v>1.148071536828287E-16</v>
+        <v>1.147825127243631E-16</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -487,7 +487,7 @@
         <v>22</v>
       </c>
       <c r="D5">
-        <v>-8.636902351770322E-17</v>
+        <v>-8.635916713431698E-17</v>
       </c>
       <c r="E5">
         <v>0.9999999999999999</v>
@@ -514,7 +514,7 @@
         <v>22</v>
       </c>
       <c r="D6">
-        <v>1.413405377585649E-17</v>
+        <v>1.41685511177083E-17</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -541,7 +541,7 @@
         <v>22</v>
       </c>
       <c r="D7">
-        <v>3.716349355778722E-17</v>
+        <v>3.722139981018134E-17</v>
       </c>
       <c r="E7">
         <v>0.9999999999999999</v>
@@ -568,7 +568,7 @@
         <v>22</v>
       </c>
       <c r="D8">
-        <v>1.513447668955902E-17</v>
+        <v>1.513694078540558E-17</v>
       </c>
       <c r="E8">
         <v>0.9999999999999999</v>
@@ -595,7 +595,7 @@
         <v>22</v>
       </c>
       <c r="D9">
-        <v>2.378776527870895E-18</v>
+        <v>2.387092851353028E-18</v>
       </c>
       <c r="E9">
         <v>0.9999999999999999</v>
@@ -622,7 +622,7 @@
         <v>22</v>
       </c>
       <c r="D10">
-        <v>1.400019176899222E-16</v>
+        <v>1.400160862410399E-16</v>
       </c>
       <c r="E10">
         <v>0.9999999999999999</v>
@@ -649,7 +649,7 @@
         <v>22</v>
       </c>
       <c r="D11">
-        <v>4.749791153825132E-17</v>
+        <v>4.752748068841002E-17</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -676,7 +676,7 @@
         <v>22</v>
       </c>
       <c r="D12">
-        <v>8.573575088513782E-17</v>
+        <v>8.57603918436034E-17</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -703,7 +703,7 @@
         <v>22</v>
       </c>
       <c r="D13">
-        <v>2.898269534721478E-17</v>
+        <v>2.899008763475445E-17</v>
       </c>
       <c r="E13">
         <v>0.9999999999999999</v>
@@ -730,7 +730,7 @@
         <v>22</v>
       </c>
       <c r="D14">
-        <v>1.064489405713041E-17</v>
+        <v>1.066368278796041E-17</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -757,7 +757,7 @@
         <v>22</v>
       </c>
       <c r="D15">
-        <v>-1.448980761370329E-17</v>
+        <v>-1.449011562568411E-17</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -784,7 +784,7 @@
         <v>22</v>
       </c>
       <c r="D16">
-        <v>-1.731766560960938E-16</v>
+        <v>-1.731618715210144E-16</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -865,7 +865,7 @@
         <v>22</v>
       </c>
       <c r="D19">
-        <v>-1.07040323574478E-17</v>
+        <v>-1.073360150760649E-17</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -892,7 +892,7 @@
         <v>22</v>
       </c>
       <c r="D20">
-        <v>-2.858351182007239E-18</v>
+        <v>-2.846646726736088E-18</v>
       </c>
       <c r="E20">
         <v>0.9999999999999999</v>
@@ -919,7 +919,7 @@
         <v>22</v>
       </c>
       <c r="D21">
-        <v>-1.2021830816187E-16</v>
+        <v>-1.202238523775247E-16</v>
       </c>
       <c r="E21">
         <v>0.9999999999999999</v>
@@ -973,7 +973,7 @@
         <v>22</v>
       </c>
       <c r="D23">
-        <v>1.548191420392369E-17</v>
+        <v>1.551148335408239E-17</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -1000,7 +1000,7 @@
         <v>22</v>
       </c>
       <c r="D24">
-        <v>3.802099891238939E-17</v>
+        <v>3.803085529577562E-17</v>
       </c>
       <c r="E24">
         <v>0.9999999999999999</v>
@@ -1027,7 +1027,7 @@
         <v>22</v>
       </c>
       <c r="D25">
-        <v>-3.244721410747528E-17</v>
+        <v>-3.245275832313003E-17</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -1054,7 +1054,7 @@
         <v>22</v>
       </c>
       <c r="D26">
-        <v>2.455717920679668E-17</v>
+        <v>2.460646112372784E-17</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -1108,7 +1108,7 @@
         <v>22</v>
       </c>
       <c r="D28">
-        <v>-1.143340472802896E-17</v>
+        <v>-1.143586882387551E-17</v>
       </c>
       <c r="E28">
         <v>0.9999999999999999</v>
@@ -1135,7 +1135,7 @@
         <v>22</v>
       </c>
       <c r="D29">
-        <v>2.056041574367966E-17</v>
+        <v>2.057027212706589E-17</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -1162,7 +1162,7 @@
         <v>22</v>
       </c>
       <c r="D30">
-        <v>5.078501539755965E-17</v>
+        <v>5.079487178094588E-17</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -1189,7 +1189,7 @@
         <v>22</v>
       </c>
       <c r="D31">
-        <v>2.848494798621007E-18</v>
+        <v>2.855887086160681E-18</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -1216,7 +1216,7 @@
         <v>22</v>
       </c>
       <c r="D32">
-        <v>9.904926074409051E-17</v>
+        <v>9.903201207316459E-17</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -1243,7 +1243,7 @@
         <v>22</v>
       </c>
       <c r="D33">
-        <v>4.918828128899009E-17</v>
+        <v>4.918396912125861E-17</v>
       </c>
       <c r="E33">
         <v>1</v>

</xml_diff>